<commit_message>
Fix USD→EUR conversion and expand dashboard by asset type
Fixes:
- Corrected GOOGLEFINANCE formula: multiply by USDEUR instead of divide

New features:
- Expanded "Composition by Type" section with: Cost, Value, P&L, Return, TIR
- Added separate flow sheets for TIR calculation by type (Crypto, Stock, ETF)
- Now 7 sheets total for comprehensive analysis
</commit_message>
<xml_diff>
--- a/dashboard_posiciones_abiertas.xlsx
+++ b/dashboard_posiciones_abiertas.xlsx
@@ -10,7 +10,10 @@
     <sheet name="Posiciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Flujos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Calendario" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Flujos_Crypto" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Flujos_Stock" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Flujos_ETF" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Calendario" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45,6 +48,7 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="002E75B6"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -453,16 +457,16 @@
   <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -543,7 +547,7 @@
         <v>18462.31</v>
       </c>
       <c r="G2" s="2">
-        <f>IFERROR(GOOGLEFINANCE("BTCUSD","price")/GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
+        <f>IFERROR(GOOGLEFINANCE("BTCUSD","price")*GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
         <v/>
       </c>
       <c r="H2" s="2">
@@ -585,7 +589,7 @@
         <v>2014.05</v>
       </c>
       <c r="G3" s="2">
-        <f>IFERROR(GOOGLEFINANCE("ETHUSD","price")/GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
+        <f>IFERROR(GOOGLEFINANCE("ETHUSD","price")*GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
         <v/>
       </c>
       <c r="H3" s="2">
@@ -627,7 +631,7 @@
         <v>139.85</v>
       </c>
       <c r="G4" s="2">
-        <f>IFERROR(GOOGLEFINANCE("SOLUSD","price")/GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
+        <f>IFERROR(GOOGLEFINANCE("SOLUSD","price")*GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
         <v/>
       </c>
       <c r="H4" s="2">
@@ -669,7 +673,7 @@
         <v>11.04</v>
       </c>
       <c r="G5" s="2">
-        <f>IFERROR(GOOGLEFINANCE("NU","price")/GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
+        <f>IFERROR(GOOGLEFINANCE("NU","price")*GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
         <v/>
       </c>
       <c r="H5" s="2">
@@ -711,7 +715,7 @@
         <v>181.13</v>
       </c>
       <c r="G6" s="2">
-        <f>IFERROR(GOOGLEFINANCE("AMZN","price")/GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
+        <f>IFERROR(GOOGLEFINANCE("AMZN","price")*GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
         <v/>
       </c>
       <c r="H6" s="2">
@@ -753,7 +757,7 @@
         <v>521.37</v>
       </c>
       <c r="G7" s="2">
-        <f>IFERROR(GOOGLEFINANCE("SPY","price")/GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
+        <f>IFERROR(GOOGLEFINANCE("SPY","price")*GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
         <v/>
       </c>
       <c r="H7" s="2">
@@ -795,7 +799,7 @@
         <v>61.11</v>
       </c>
       <c r="G8" s="2">
-        <f>IFERROR(GOOGLEFINANCE("IEV","price")/GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
+        <f>IFERROR(GOOGLEFINANCE("IEV","price")*GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
         <v/>
       </c>
       <c r="H8" s="2">
@@ -837,7 +841,7 @@
         <v>84.81</v>
       </c>
       <c r="G9" s="2">
-        <f>IFERROR(GOOGLEFINANCE("ARGT","price")/GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
+        <f>IFERROR(GOOGLEFINANCE("ARGT","price")*GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
         <v/>
       </c>
       <c r="H9" s="2">
@@ -879,7 +883,7 @@
         <v>261.59</v>
       </c>
       <c r="G10" s="2">
-        <f>IFERROR(GOOGLEFINANCE("AAPL","price")/GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
+        <f>IFERROR(GOOGLEFINANCE("AAPL","price")*GOOGLEFINANCE("CURRENCY:USDEUR"),0)</f>
         <v/>
       </c>
       <c r="H10" s="2">
@@ -929,11 +933,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -962,156 +970,298 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Coste Total</t>
-        </is>
-      </c>
-      <c r="B5" s="2">
-        <f>Posiciones!E11</f>
-        <v/>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Métrica</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Valor Actual</t>
+          <t>Coste Total</t>
         </is>
       </c>
       <c r="B6" s="2">
-        <f>Posiciones!H11</f>
+        <f>Posiciones!E11</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>P&amp;L</t>
+          <t>Valor Actual</t>
         </is>
       </c>
       <c r="B7" s="2">
-        <f>Posiciones!I11</f>
+        <f>Posiciones!H11</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="B8" s="3">
-        <f>Posiciones!J11</f>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+      <c r="B8" s="2">
+        <f>Posiciones!I11</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Rentabilidad</t>
+        </is>
+      </c>
+      <c r="B9" s="3">
+        <f>Posiciones!J11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>TIR Anualizada</t>
         </is>
       </c>
-      <c r="B9" s="3">
+      <c r="B10" s="3">
         <f>IFERROR(XIRR(Flujos!B:B,Flujos!A:A),0)</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>COMPOSICIÓN POR TIPO</t>
-        </is>
-      </c>
-    </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>COMPOSICIÓN POR TIPO DE ACTIVO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Valor (€)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Crypto</t>
-        </is>
-      </c>
-      <c r="B14">
-        <f>SUMIF(Posiciones!C:C,"Crypto",Posiciones!H:H)</f>
-        <v/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Coste (€)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Valor Actual (€)</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>P&amp;L (€)</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Retorno Simple</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>TIR</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="B15">
-        <f>SUMIF(Posiciones!C:C,"Stock",Posiciones!H:H)</f>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="B15" s="2">
+        <f>SUMIF(Posiciones!C:C,"Crypto",Posiciones!E:E)</f>
+        <v/>
+      </c>
+      <c r="C15" s="2">
+        <f>SUMIF(Posiciones!C:C,"Crypto",Posiciones!H:H)</f>
+        <v/>
+      </c>
+      <c r="D15" s="2">
+        <f>C15-B15</f>
+        <v/>
+      </c>
+      <c r="E15" s="3">
+        <f>IF(B15&gt;0,D15/B15,0)</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>IFERROR(XIRR(Flujos_Crypto!B:B,Flujos_Crypto!A:A),"-")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <f>SUMIF(Posiciones!C:C,"Stock",Posiciones!E:E)</f>
+        <v/>
+      </c>
+      <c r="C16" s="2">
+        <f>SUMIF(Posiciones!C:C,"Stock",Posiciones!H:H)</f>
+        <v/>
+      </c>
+      <c r="D16" s="2">
+        <f>C16-B16</f>
+        <v/>
+      </c>
+      <c r="E16" s="3">
+        <f>IF(B16&gt;0,D16/B16,0)</f>
+        <v/>
+      </c>
+      <c r="F16">
+        <f>IFERROR(XIRR(Flujos_Stock!B:B,Flujos_Stock!A:A),"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="B16">
+      <c r="B17" s="2">
+        <f>SUMIF(Posiciones!C:C,"ETF",Posiciones!E:E)</f>
+        <v/>
+      </c>
+      <c r="C17" s="2">
         <f>SUMIF(Posiciones!C:C,"ETF",Posiciones!H:H)</f>
         <v/>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="D17" s="2">
+        <f>C17-B17</f>
+        <v/>
+      </c>
+      <c r="E17" s="3">
+        <f>IF(B17&gt;0,D17/B17,0)</f>
+        <v/>
+      </c>
+      <c r="F17">
+        <f>IFERROR(XIRR(Flujos_ETF!B:B,Flujos_ETF!A:A),"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <f>SUM(B15:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="2">
+        <f>SUM(C15:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="2">
+        <f>SUM(D15:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="3">
+        <f>IF(B18&gt;0,D18/B18,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>COMPOSICIÓN POR BROKER</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>Broker</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Valor (€)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Coste (€)</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Valor Actual (€)</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>P&amp;L (€)</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Retorno Simple</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Kraken</t>
         </is>
       </c>
-      <c r="B21">
+      <c r="B23" s="2">
+        <f>SUMIF(Posiciones!B:B,"Kraken",Posiciones!E:E)</f>
+        <v/>
+      </c>
+      <c r="C23" s="2">
         <f>SUMIF(Posiciones!B:B,"Kraken",Posiciones!H:H)</f>
         <v/>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="D23" s="2">
+        <f>C23-B23</f>
+        <v/>
+      </c>
+      <c r="E23" s="3">
+        <f>IF(B23&gt;0,D23/B23,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Fintual</t>
         </is>
       </c>
-      <c r="B22">
+      <c r="B24" s="2">
+        <f>SUMIF(Posiciones!B:B,"Fintual",Posiciones!E:E)</f>
+        <v/>
+      </c>
+      <c r="C24" s="2">
         <f>SUMIF(Posiciones!B:B,"Fintual",Posiciones!H:H)</f>
+        <v/>
+      </c>
+      <c r="D24" s="2">
+        <f>C24-B24</f>
+        <v/>
+      </c>
+      <c r="E24" s="3">
+        <f>IF(B24&gt;0,D24/B24,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1123,12 +1273,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1147,6 +1298,11 @@
           <t>Concepto</t>
         </is>
       </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1162,6 +1318,11 @@
           <t>Compra BTC</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1177,6 +1338,11 @@
           <t>Compra BTC</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1192,6 +1358,11 @@
           <t>Compra ETH</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1207,6 +1378,11 @@
           <t>Compra SOL</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1222,6 +1398,11 @@
           <t>Compra BTC</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1237,6 +1418,11 @@
           <t>Compra BTC</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1252,6 +1438,11 @@
           <t>Compra ETH</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1267,6 +1458,11 @@
           <t>Compra SOL</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1282,6 +1478,11 @@
           <t>Compra BTC</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1297,6 +1498,11 @@
           <t>Compra ETH</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1312,6 +1518,11 @@
           <t>Compra BTC</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1327,6 +1538,11 @@
           <t>Compra NU</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1342,6 +1558,11 @@
           <t>Compra NU</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1357,6 +1578,11 @@
           <t>Compra AMZN</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1372,6 +1598,11 @@
           <t>Compra SPY</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ETF</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1387,6 +1618,11 @@
           <t>Compra NU</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1402,6 +1638,11 @@
           <t>Compra IEV</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ETF</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1417,6 +1658,11 @@
           <t>Compra ARGT</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ETF</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1432,6 +1678,11 @@
           <t>Compra AMZN</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1445,6 +1696,11 @@
       <c r="C21" t="inlineStr">
         <is>
           <t>Compra AAPL</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
     </row>
@@ -1469,6 +1725,314 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Flujo (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2020-05-19</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>-248</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2021-05-19</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>-250</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2021-05-19</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>-250</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2021-12-03</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>-200</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2022-01-25</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>-196.46</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2022-01-25</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>-3.83</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2022-01-25</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>-300.75</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2022-01-25</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>-98.95</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2023-02-02</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>-150</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2023-02-02</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>-150</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2023-04-23</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>-200</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <f>TODAY()</f>
+        <v/>
+      </c>
+      <c r="B13" s="2">
+        <f>SUMIF(Posiciones!C:C,"Crypto",Posiciones!H:H)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Flujo (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>-576.92</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>-192.31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>-480.77</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>-240.38</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>-605.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>-1193.89</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <f>TODAY()</f>
+        <v/>
+      </c>
+      <c r="B8" s="2">
+        <f>SUMIF(Posiciones!C:C,"Stock",Posiciones!H:H)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Flujo (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>-240.38</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>-1255.4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>-1356.09</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <f>TODAY()</f>
+        <v/>
+      </c>
+      <c r="B5" s="2">
+        <f>SUMIF(Posiciones!C:C,"ETF",Posiciones!H:H)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>